<commit_message>
one more cycle of validation
</commit_message>
<xml_diff>
--- a/tests/TeamworkDB/output/utilization_failures_report_202605.xlsx
+++ b/tests/TeamworkDB/output/utilization_failures_report_202605.xlsx
@@ -598,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -924,7 +924,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>CRNY</t>
+          <t>CRSV</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -939,29 +939,29 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>971.30</t>
+          <t>339.20</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>1,083.80</t>
+          <t>367.50</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>112.50</t>
+          <t>28.30</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>11.58%</t>
+          <t>8.34%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>CRSV</t>
+          <t>CRCH</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -971,39 +971,39 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Actual_Hours</t>
+          <t>Standard_Rev</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>339.20</t>
+          <t>736,416.00</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>367.50</t>
+          <t>800,506.00</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>28.30</t>
+          <t>64,090.00</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>8.34%</t>
+          <t>8.70%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>CRCH</t>
+          <t>CRDC</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Officer</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1013,29 +1013,29 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>736,416.00</t>
+          <t>3,707,951.00</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>800,506.00</t>
+          <t>3,579,746.00</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>64,090.00</t>
+          <t>128,205.00</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>3.46%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>CRDC</t>
+          <t>CRNY</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1050,178 +1050,178 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>3,707,951.00</t>
+          <t>3,201,489.50</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>3,579,746.00</t>
+          <t>3,329,695.00</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>128,205.00</t>
+          <t>128,205.50</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>3.46%</t>
+          <t>4.00%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>CRSV</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Officer</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Standard_Rev</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>431,386.00</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>471,006.00</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>39,620.00</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>9.18%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: 2026_US (YTD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Util Report</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Diff%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>CRDC</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Target_Hours</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>18,937.86</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>18,182.90</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>754.96</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>3.99%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>CRNY</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Standard_Rev</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>3,201,489.50</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>3,329,695.00</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>128,205.50</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>4.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>CRNY</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Officer</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Standard_Rev</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>1,248,464.50</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>1,384,590.00</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>136,125.50</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>10.90%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>CRSV</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Officer</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Standard_Rev</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>431,386.00</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>471,006.00</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>39,620.00</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>9.18%</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Sheet: 2026_US (YTD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Office</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Util Report</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Diff</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Diff%</t>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Target_Hours</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>16,762.83</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>17,517.80</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>754.97</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>4.50%</t>
         </is>
       </c>
     </row>
@@ -1238,27 +1238,27 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Target_Hours</t>
+          <t>Target_Rev</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>18,937.86</t>
+          <t>18,587,971.28</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>18,182.90</t>
+          <t>17,889,606.00</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>754.96</t>
+          <t>698,365.28</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>3.99%</t>
+          <t>3.76%</t>
         </is>
       </c>
     </row>
@@ -1275,71 +1275,71 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Target_Hours</t>
+          <t>Target_Rev</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>16,762.83</t>
+          <t>16,197,153.70</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>17,517.80</t>
+          <t>16,895,519.00</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>754.97</t>
+          <t>698,365.30</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>4.31%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>CRDC</t>
+          <t>CRCH</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Officer</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Target_Rev</t>
+          <t>Actual_Hours</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>18,587,971.28</t>
+          <t>3,335.50</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>17,889,606.00</t>
+          <t>3,644.50</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>698,365.28</t>
+          <t>309.00</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>3.76%</t>
+          <t>9.26%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>CRNY</t>
+          <t>CRDC</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1349,39 +1349,39 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Target_Rev</t>
+          <t>Actual_Hours</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>16,197,153.70</t>
+          <t>19,126.10</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>16,895,519.00</t>
+          <t>18,449.00</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>698,365.30</t>
+          <t>677.10</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>4.31%</t>
+          <t>3.54%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>CRCH</t>
+          <t>CRNY</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Officer</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -1391,34 +1391,34 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>3,335.50</t>
+          <t>16,738.00</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>3,644.50</t>
+          <t>17,415.10</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>309.00</t>
+          <t>677.10</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>9.26%</t>
+          <t>4.05%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>CRDC</t>
+          <t>CRSV</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Officer</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1428,108 +1428,108 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>19,126.10</t>
+          <t>1,385.10</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>18,449.00</t>
+          <t>1,575.70</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>677.10</t>
+          <t>190.60</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>3.54%</t>
+          <t>13.76%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>CRNY</t>
+          <t>CRCH</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Officer</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Actual_Hours</t>
+          <t>Standard_Rev</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>16,738.00</t>
+          <t>4,266,630.00</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>17,415.10</t>
+          <t>4,714,680.00</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>677.10</t>
+          <t>448,050.00</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>4.05%</t>
+          <t>10.50%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>CRSV</t>
+          <t>CRDC</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Officer</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Actual_Hours</t>
+          <t>Standard_Rev</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>1,385.10</t>
+          <t>18,677,073.00</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>1,575.70</t>
+          <t>18,050,756.00</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>190.60</t>
+          <t>626,317.00</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>13.76%</t>
+          <t>3.35%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>CRCH</t>
+          <t>CRNY</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Officer</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -1539,34 +1539,34 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>4,266,630.00</t>
+          <t>16,388,163.50</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>4,714,680.00</t>
+          <t>17,014,481.00</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>448,050.00</t>
+          <t>626,317.50</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>10.50%</t>
+          <t>3.82%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>CRDC</t>
+          <t>CRSV</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Officer</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -1576,94 +1576,20 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>18,677,073.00</t>
+          <t>1,775,144.00</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>18,050,756.00</t>
+          <t>2,041,984.00</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>626,317.00</t>
+          <t>266,840.00</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>3.35%</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>CRNY</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Manager</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Standard_Rev</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>16,388,163.50</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>17,014,481.00</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>626,317.50</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>3.82%</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>CRSV</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Officer</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Standard_Rev</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>1,775,144.00</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>2,041,984.00</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>266,840.00</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>15.03%</t>
         </is>
@@ -1684,12 +1610,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="33" customWidth="1" min="5" max="5"/>
     <col width="33" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1829,12 +1755,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>5674</t>
+          <t>1379</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Li Bergolis, Matteo</t>
+          <t>Bickford, Eric</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1844,34 +1770,34 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>11.80</t>
+          <t>28.40</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>124.30</t>
+          <t>29.60</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>112.50</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>953.39%</t>
+          <t>4.23%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>5674</t>
+          <t>1379</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Li Bergolis, Matteo</t>
+          <t>Bickford, Eric</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1881,22 +1807,22 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>14,278.00</t>
+          <t>35,926.00</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>150,403.00</t>
+          <t>37,444.00</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>136,125.00</t>
+          <t>1,518.00</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>953.39%</t>
+          <t>4.23%</t>
         </is>
       </c>
     </row>
@@ -2085,16 +2011,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="33" customWidth="1" min="5" max="5"/>
     <col width="33" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2108,7 +2034,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Sheet: YTD - CRNY (YTD)</t>
+          <t>Sheet: YTD - CRSF (YTD)</t>
         </is>
       </c>
     </row>
@@ -2152,12 +2078,12 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>5674</t>
+          <t>101650</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Li Bergolis, Matteo</t>
+          <t>Li, Lily</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -2167,313 +2093,246 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>582.80</t>
+          <t>165.70</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>695.30</t>
+          <t>170.70</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>112.50</t>
+          <t>5.00</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>19.30%</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>5674</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Li Bergolis, Matteo</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Standard_Rev</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>705,188.00</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>841,313.00</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>136,125.00</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>19.30%</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Sheet: YTD - CRSF (YTD)</t>
-        </is>
-      </c>
-    </row>
+          <t>3.02%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>MISSING ROWS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: YTD - CRDC (YTD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>EmpNo</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Util Report</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Diff</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Diff%</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>101650</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Li, Lily</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Actual_Hours</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>165.70</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>170.70</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>5.00</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>3.02%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>MISSING ROWS</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>MISSING IN DB</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>102231</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Conell-Price, Lynn</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Employee_name: Conell-Price, Lynn</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>OFFC: CRNY</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Total_Billable_Hours: 138.6000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: DC</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Sheet: YTD - CRDC (YTD)</t>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>EmpNo</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>MISSING IN DB</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>102231</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Conell-Price, Lynn</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Employee_name: Conell-Price, Lynn</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>OFFC: CRNY</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Total_Billable_Hours: 138.6000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: YTD - CRNY (YTD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>EmpNo</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>MISSING IN DB</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MISSING IN XLS</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>102231</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Conell-Price, Lynn</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Employee_name: Conell-Price, Lynn</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>OFFC: CRNY</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>Total_Billable_Hours: 138.6000</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Sheet: DC</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Target_Hrs: 139.27</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Actual_Hrs: 138.60000000000002</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: NY</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>EmpNo</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>MISSING IN DB</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>MISSING IN XLS</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>102231</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Conell-Price, Lynn</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Employee_name: Conell-Price, Lynn</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>OFFC: CRNY</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>Total_Billable_Hours: 138.6000</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Sheet: YTD - CRNY (YTD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>EmpNo</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>MISSING IN XLS</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>102231</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Target_Hrs: 139.27</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Actual_Hrs: 138.60000000000002</t>
         </is>

</xml_diff>